<commit_message>
整合UnitConfig Monster Hero Entity
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/__tables__.xlsx
+++ b/Design/Excel/ET/Datas/__tables__.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\ugit\myGameDevelopmentKit\Design\Excel\ET\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABB15EB-C410-4F05-A7F0-95D4D218C730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85094238-C85E-40BB-B8D2-A981646E5420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="1140" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="19200" windowHeight="9970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
   <si>
     <t>##var</t>
   </si>
@@ -235,6 +235,7 @@
         <sz val="11"/>
         <color rgb="FF800080"/>
         <rFont val="等线"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -246,6 +247,7 @@
         <sz val="11"/>
         <color rgb="FF800080"/>
         <rFont val="等线"/>
+        <family val="3"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
@@ -274,9 +276,6 @@
     <t>DRUnitConfig</t>
   </si>
   <si>
-    <t>UnitConfig.xlsx</t>
-  </si>
-  <si>
     <t>c</t>
   </si>
   <si>
@@ -316,15 +315,31 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>DTUnit</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>DRUnit</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>Game/Unit.xlsx</t>
+    <t>Game/Hero.xlsx</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>DTHero</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRHero</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>DTMonster</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>DRMonster</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Game/Monster.xlsx</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Game/UnitConfig.xlsx</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -344,6 +359,7 @@
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -352,6 +368,7 @@
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -360,6 +377,7 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -367,12 +385,14 @@
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -724,12 +744,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29.08203125" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="58.33203125" customWidth="1"/>
+    <col min="4" max="4" width="27.1640625" customWidth="1"/>
     <col min="5" max="5" width="24.33203125" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" customWidth="1"/>
     <col min="7" max="7" width="11.25" customWidth="1"/>
@@ -1075,8 +1095,8 @@
       <c r="D17" t="b">
         <v>1</v>
       </c>
-      <c r="E17" t="s">
-        <v>73</v>
+      <c r="E17" s="6" t="s">
+        <v>89</v>
       </c>
       <c r="H17" t="s">
         <v>67</v>
@@ -1084,53 +1104,53 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D18" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="H18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D19" t="b">
-        <v>1</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="H19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="H20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
@@ -1144,10 +1164,27 @@
         <v>1</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B22" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="H21" t="s">
-        <v>74</v>
+      <c r="C22" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H22" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add skill attribute config table
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/__tables__.xlsx
+++ b/Design/Excel/ET/Datas/__tables__.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="29.08203125" customWidth="1" style="7" min="2" max="2"/>
@@ -1194,75 +1194,100 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>DTSkillCardRule</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>DRSkillCardRule</t>
         </is>
       </c>
-      <c r="D25" t="b">
-        <v>1</v>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="D25" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>Game/SkillCardRule.xlsx</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="0" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>DTBattleCardConfig</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>DRBattleCardConfig</t>
         </is>
       </c>
-      <c r="D26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="D26" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>Game/BattleCardConfig.xlsx</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="0" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>DTRelic</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>DRRelic</t>
         </is>
       </c>
-      <c r="D27" t="b">
-        <v>1</v>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D27" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>Game/Relic.xlsx</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="0" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DTSkillAttribute</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>DRSkillAttribute</t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Game/SkillAttribute.xlsx</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>c</t>
         </is>

</xml_diff>